<commit_message>
refactor(equity): strengthen exchange scoping and unwind correctness
- eliminate rounding drift during loop recapture and terminal settlement
- distinguish genuine forward surface from rounding-only remainder
- preserve exact tracked quantities during recapture and residual carry-back
- prevent already-recognized residuals from being re-terminalized
- require explicit ExchangeTarget scoping for every exchange
- support separate exchange accounts for from/to legs
- remove implicit universal exchange-account mode
- extract EventBuilder from Ledger and expand scenario infrastructure
- add comprehensive unwind scenarios and invariants for rounding, residuals, and intermediate hops
- update architecture documentation for exchange targets, residual settlement, and unwind semantics
</commit_message>
<xml_diff>
--- a/example/account-ledger.xlsx
+++ b/example/account-ledger.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Local Storage\Repositories\Finance\Lattice\example\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{453BAD59-C8AE-472C-BDF9-F583EAB00AB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50846043-FBC4-405B-82BC-47A9741CB15C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="51495" yWindow="3420" windowWidth="19410" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="70695" yWindow="3420" windowWidth="19410" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="12">
   <si>
     <t>Cash</t>
   </si>
@@ -78,7 +78,22 @@
     <t>B (Currency)</t>
   </si>
   <si>
-    <t>Foreign Exchange Expense</t>
+    <t>Exchange Expense</t>
+  </si>
+  <si>
+    <t>C (Inventory)</t>
+  </si>
+  <si>
+    <t>Rent Expense</t>
+  </si>
+  <si>
+    <t>Spoilage Expense</t>
+  </si>
+  <si>
+    <t>Inventory</t>
+  </si>
+  <si>
+    <t>Profit from Sale of Inventory</t>
   </si>
 </sst>
 </file>
@@ -410,16 +425,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:H42"/>
+  <dimension ref="B1:L42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="43.5703125" customWidth="1"/>
     <col min="3" max="4" width="13" customWidth="1"/>
     <col min="6" max="6" width="43.5703125" customWidth="1"/>
     <col min="7" max="8" width="13" customWidth="1"/>
+    <col min="10" max="10" width="43.5703125" customWidth="1"/>
+    <col min="11" max="12" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B1" s="2" t="s">
         <v>4</v>
       </c>
@@ -430,8 +447,13 @@
       </c>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-    </row>
-    <row r="2" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="J1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="K1" s="2"/>
+      <c r="L1" s="2"/>
+    </row>
+    <row r="2" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>0</v>
       </c>
@@ -445,8 +467,14 @@
         <f>H3</f>
         <v>250</v>
       </c>
-    </row>
-    <row r="3" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="J2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K2">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="3" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
@@ -461,8 +489,15 @@
         <f>C5*0.5</f>
         <v>250</v>
       </c>
-    </row>
-    <row r="5" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="J3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="L3">
+        <f>K2</f>
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>2</v>
       </c>
@@ -477,8 +512,14 @@
         <f>H6</f>
         <v>250</v>
       </c>
-    </row>
-    <row r="6" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="J5" t="s">
+        <v>2</v>
+      </c>
+      <c r="K5">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B6" s="1" t="s">
         <v>0</v>
       </c>
@@ -491,8 +532,15 @@
       <c r="H6">
         <v>250</v>
       </c>
-    </row>
-    <row r="8" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="J6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L6">
+        <f>K5</f>
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>0</v>
       </c>
@@ -507,7 +555,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="9" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B9" s="1" t="s">
         <v>2</v>
       </c>
@@ -519,11 +567,12 @@
         <v>2</v>
       </c>
       <c r="H9">
-        <f>C12*0.5</f>
+        <f>C13*0.5</f>
         <v>500</v>
       </c>
-    </row>
-    <row r="10" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="J9" s="1"/>
+    </row>
+    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B10" s="1" t="s">
         <v>3</v>
       </c>
@@ -532,24 +581,38 @@
         <v>50</v>
       </c>
     </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="F11" t="s">
+        <v>2</v>
+      </c>
+      <c r="G11">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C12">
-        <f>(C2-D6)+500</f>
+        <v>50</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="H12">
+        <f>G11</f>
+        <v>200</v>
+      </c>
+    </row>
+    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
+        <v>2</v>
+      </c>
+      <c r="C13">
         <v>1000</v>
       </c>
     </row>
-    <row r="13" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B13" t="s">
-        <v>6</v>
-      </c>
-      <c r="C13">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="14" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B14" s="1" t="s">
         <v>0</v>
       </c>
@@ -557,104 +620,223 @@
         <f>SUM(C12:C13)</f>
         <v>1050</v>
       </c>
-    </row>
-    <row r="34" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="F14" t="s">
+        <v>2</v>
+      </c>
+      <c r="G14">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="F15" t="s">
+        <v>2</v>
+      </c>
+      <c r="G15">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="16" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B16" t="s">
+        <v>8</v>
+      </c>
+      <c r="C16">
+        <f>D17</f>
+        <v>400</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="H16">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="17" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B17" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D17">
+        <f>G11*2</f>
+        <v>400</v>
+      </c>
+    </row>
+    <row r="18" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="F18" t="s">
+        <v>0</v>
+      </c>
+      <c r="G18">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="19" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B19" t="s">
+        <v>9</v>
+      </c>
+      <c r="C19">
+        <f>D20</f>
+        <v>100</v>
+      </c>
+      <c r="F19" t="s">
+        <v>11</v>
+      </c>
+      <c r="H19">
+        <f>G18-H20</f>
+        <v>150</v>
+      </c>
+    </row>
+    <row r="20" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B20" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D20">
+        <f>G14*2</f>
+        <v>100</v>
+      </c>
+      <c r="F20" t="s">
+        <v>2</v>
+      </c>
+      <c r="H20">
+        <f>G15*(K5/L3)</f>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="34" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B34" t="str" cm="1">
-        <f t="array" ref="B34:B37">_xlfn.LET(_xlpm.x,_xlfn.UNIQUE($B$5:$B$33),_xlfn._xlws.FILTER(_xlpm.x,_xlpm.x&lt;&gt;0))</f>
-        <v>Net Transfers</v>
+        <f t="array" ref="B34:B40">_xlfn.LET(_xlpm.x,_xlfn.UNIQUE(B$2:B$33),_xlfn._xlws.FILTER(_xlpm.x,_xlpm.x&lt;&gt;0))</f>
+        <v>Cash</v>
       </c>
       <c r="D34" cm="1">
         <f t="array" ref="D34">SUMPRODUCT(--(B34=B$2:B$33),C$2:C$33-D$2:D$33)</f>
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="F34" t="str" cm="1">
-        <f t="array" ref="F34:F37">_xlfn.LET(_xlpm.x,_xlfn.UNIQUE($B$5:$B$33),_xlfn._xlws.FILTER(_xlpm.x,_xlpm.x&lt;&gt;0))</f>
-        <v>Net Transfers</v>
+        <f t="array" ref="F34:F36">_xlfn.LET(_xlpm.x,_xlfn.UNIQUE(F$2:F$33),_xlfn._xlws.FILTER(_xlpm.x,_xlpm.x&lt;&gt;0))</f>
+        <v>Cash</v>
       </c>
       <c r="H34" cm="1">
         <f t="array" ref="H34">SUMPRODUCT(--(F34=F$2:F$33),G$2:G$33-H$2:H$33)</f>
-        <v>-500</v>
-      </c>
-    </row>
-    <row r="35" spans="2:8" x14ac:dyDescent="0.25">
+        <v>250</v>
+      </c>
+      <c r="J34" t="str" cm="1">
+        <f t="array" ref="J34:J35">_xlfn.LET(_xlpm.x,_xlfn.UNIQUE(J$2:J$33),_xlfn._xlws.FILTER(_xlpm.x,_xlpm.x&lt;&gt;0))</f>
+        <v>Inventory</v>
+      </c>
+      <c r="L34" cm="1">
+        <f t="array" ref="L34">SUMPRODUCT(--(J34=J$2:J$33),K$2:K$33-L$2:L$33)</f>
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="35" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B35" t="str">
-        <v>Cash</v>
+        <v>Opening Balance</v>
       </c>
       <c r="D35" cm="1">
         <f t="array" ref="D35">SUMPRODUCT(--(B35=B$2:B$33),C$2:C$33-D$2:D$33)</f>
-        <v>0</v>
+        <v>-1000</v>
       </c>
       <c r="F35" t="str">
-        <v>Cash</v>
+        <v>Net Transfers</v>
       </c>
       <c r="H35" cm="1">
         <f t="array" ref="H35">SUMPRODUCT(--(F35=F$2:F$33),G$2:G$33-H$2:H$33)</f>
-        <v>500</v>
-      </c>
-    </row>
-    <row r="36" spans="2:8" x14ac:dyDescent="0.25">
+        <v>-100</v>
+      </c>
+      <c r="J35" t="str">
+        <v>Net Transfers</v>
+      </c>
+      <c r="L35" cm="1">
+        <f t="array" ref="L35">SUMPRODUCT(--(J35=J$2:J$33),K$2:K$33-L$2:L$33)</f>
+        <v>-3000</v>
+      </c>
+    </row>
+    <row r="36" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B36" t="str">
-        <v>Capital Gains or Losses</v>
+        <v>Net Transfers</v>
       </c>
       <c r="D36" cm="1">
         <f t="array" ref="D36">SUMPRODUCT(--(B36=B$2:B$33),C$2:C$33-D$2:D$33)</f>
-        <v>-50</v>
+        <v>500</v>
       </c>
       <c r="F36" t="str">
-        <v>Capital Gains or Losses</v>
+        <v>Profit from Sale of Inventory</v>
       </c>
       <c r="H36" cm="1">
         <f t="array" ref="H36">SUMPRODUCT(--(F36=F$2:F$33),G$2:G$33-H$2:H$33)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" spans="2:8" x14ac:dyDescent="0.25">
+        <v>-150</v>
+      </c>
+      <c r="L36" cm="1">
+        <f t="array" ref="L36">SUMPRODUCT(--(J36=J$2:J$33),K$2:K$33-L$2:L$33)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B37" t="str">
-        <v>Foreign Exchange Expense</v>
+        <v>Capital Gains or Losses</v>
       </c>
       <c r="D37" cm="1">
         <f t="array" ref="D37">SUMPRODUCT(--(B37=B$2:B$33),C$2:C$33-D$2:D$33)</f>
-        <v>50</v>
-      </c>
-      <c r="F37" t="str">
-        <v>Foreign Exchange Expense</v>
+        <v>-50</v>
       </c>
       <c r="H37" cm="1">
         <f t="array" ref="H37">SUMPRODUCT(--(F37=F$2:F$33),G$2:G$33-H$2:H$33)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="38" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="L37" cm="1">
+        <f t="array" ref="L37">SUMPRODUCT(--(J37=J$2:J$33),K$2:K$33-L$2:L$33)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B38" t="str">
+        <v>Exchange Expense</v>
+      </c>
       <c r="D38" cm="1">
         <f t="array" ref="D38">SUMPRODUCT(--(B38=B$2:B$33),C$2:C$33-D$2:D$33)</f>
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="H38" cm="1">
         <f t="array" ref="H38">SUMPRODUCT(--(F38=F$2:F$33),G$2:G$33-H$2:H$33)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="39" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="L38" cm="1">
+        <f t="array" ref="L38">SUMPRODUCT(--(J38=J$2:J$33),K$2:K$33-L$2:L$33)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B39" t="str">
+        <v>Rent Expense</v>
+      </c>
       <c r="D39" cm="1">
         <f t="array" ref="D39">SUMPRODUCT(--(B39=B$2:B$33),C$2:C$33-D$2:D$33)</f>
-        <v>0</v>
+        <v>400</v>
       </c>
       <c r="H39" cm="1">
         <f t="array" ref="H39">SUMPRODUCT(--(F39=F$2:F$33),G$2:G$33-H$2:H$33)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="40" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="L39" cm="1">
+        <f t="array" ref="L39">SUMPRODUCT(--(J39=J$2:J$33),K$2:K$33-L$2:L$33)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B40" t="str">
+        <v>Spoilage Expense</v>
+      </c>
       <c r="D40" cm="1">
         <f t="array" ref="D40">SUMPRODUCT(--(B40=B$2:B$33),C$2:C$33-D$2:D$33)</f>
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H40" cm="1">
         <f t="array" ref="H40">SUMPRODUCT(--(F40=F$2:F$33),G$2:G$33-H$2:H$33)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="41" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="L40" cm="1">
+        <f t="array" ref="L40">SUMPRODUCT(--(J40=J$2:J$33),K$2:K$33-L$2:L$33)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="2:12" x14ac:dyDescent="0.25">
       <c r="D41" cm="1">
         <f t="array" ref="D41">SUMPRODUCT(--(B41=B$2:B$33),C$2:C$33-D$2:D$33)</f>
         <v>0</v>
@@ -663,8 +845,12 @@
         <f t="array" ref="H41">SUMPRODUCT(--(F41=F$2:F$33),G$2:G$33-H$2:H$33)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="42" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="L41" cm="1">
+        <f t="array" ref="L41">SUMPRODUCT(--(J41=J$2:J$33),K$2:K$33-L$2:L$33)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="2:12" x14ac:dyDescent="0.25">
       <c r="D42" cm="1">
         <f t="array" ref="D42">SUMPRODUCT(--(B42=B$2:B$33),C$2:C$33-D$2:D$33)</f>
         <v>0</v>
@@ -673,11 +859,16 @@
         <f t="array" ref="H42">SUMPRODUCT(--(F42=F$2:F$33),G$2:G$33-H$2:H$33)</f>
         <v>0</v>
       </c>
+      <c r="L42" cm="1">
+        <f t="array" ref="L42">SUMPRODUCT(--(J42=J$2:J$33),K$2:K$33-L$2:L$33)</f>
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="B1:D1"/>
     <mergeCell ref="F1:H1"/>
+    <mergeCell ref="J1:L1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
refactor!: redesign exchange accounting and lineage attribution
- replace proportional lineage attribution with settlement-aware forward weighting
- fix phantom exchange lineage during loop recapture (INV8)
- separate exchange and residual transaction primitives
- support dynamic account display names and orientation summaries
- expand scenario ledger with richer account hierarchy and exchange structure
- add regression coverage for settlement-aware lineage attribution
- reorganize transaction and equity infrastructure
</commit_message>
<xml_diff>
--- a/example/account-ledger.xlsx
+++ b/example/account-ledger.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Local Storage\Repositories\Finance\Lattice\example\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50846043-FBC4-405B-82BC-47A9741CB15C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73C0B67D-8071-4D6A-8DBE-5F5E29633735}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="70695" yWindow="3420" windowWidth="19410" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="52005" yWindow="4050" windowWidth="18285" windowHeight="14550" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,8 +37,9 @@
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
 <metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
+  <metadataTypes count="2">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+    <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
   </metadataTypes>
   <futureMetadata name="XLDAPR" count="1">
     <bk>
@@ -49,27 +50,45 @@
       </extLst>
     </bk>
   </futureMetadata>
+  <futureMetadata name="XLRICHVALUE" count="2">
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="0"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="1"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
   <cellMetadata count="1">
     <bk>
       <rc t="1" v="0"/>
     </bk>
   </cellMetadata>
+  <valueMetadata count="2">
+    <bk>
+      <rc t="2" v="0"/>
+    </bk>
+    <bk>
+      <rc t="2" v="1"/>
+    </bk>
+  </valueMetadata>
 </metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="9">
   <si>
     <t>Cash</t>
   </si>
   <si>
     <t>Opening Balance</t>
-  </si>
-  <si>
-    <t>Net Transfers</t>
-  </si>
-  <si>
-    <t>Capital Gains or Losses</t>
   </si>
   <si>
     <t>A (Currency)</t>
@@ -78,22 +97,19 @@
     <t>B (Currency)</t>
   </si>
   <si>
-    <t>Exchange Expense</t>
-  </si>
-  <si>
     <t>C (Inventory)</t>
   </si>
   <si>
-    <t>Rent Expense</t>
+    <t>Net Transfers</t>
   </si>
   <si>
-    <t>Spoilage Expense</t>
+    <t>Capital Gains</t>
   </si>
   <si>
-    <t>Inventory</t>
+    <t>Accounts Payable</t>
   </si>
   <si>
-    <t>Profit from Sale of Inventory</t>
+    <t>Capital Loss</t>
   </si>
 </sst>
 </file>
@@ -137,13 +153,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" indent="2"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -160,6 +179,72 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
+<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
+  <global>
+    <keyFlags>
+      <key name="_Self">
+        <flag name="ExcludeFromFile" value="1"/>
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_DisplayString">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Flags">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Format">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_SubLabel">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Attribution">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Icon">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Display">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_CanonicalPropertyNames">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_ClassificationId">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+    </keyFlags>
+  </global>
+</rvTypesInfo>
+</file>
+
+<file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="2">
+  <rv s="0">
+    <v>13</v>
+    <v>3</v>
+  </rv>
+  <rv s="1">
+    <v>13</v>
+    <v>1</v>
+  </rv>
+</rvData>
+</file>
+
+<file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
+<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="2">
+  <s t="_error">
+    <k n="errorType" t="i"/>
+    <k n="subType" t="i"/>
+  </s>
+  <s t="_error">
+    <k n="errorType" t="i"/>
+    <k n="propagated" t="b"/>
+  </s>
+</rvStructures>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -438,17 +523,17 @@
   <sheetData>
     <row r="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B1" s="2" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
       <c r="F1" s="2" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
       <c r="J1" s="2" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="K1" s="2"/>
       <c r="L1" s="2"/>
@@ -464,14 +549,7 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <f>H3</f>
-        <v>250</v>
-      </c>
-      <c r="J2" t="s">
-        <v>10</v>
-      </c>
-      <c r="K2">
-        <v>5000</v>
+        <v>250</v>
       </c>
     </row>
     <row r="3" spans="2:12" x14ac:dyDescent="0.25">
@@ -483,40 +561,26 @@
         <v>1000</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H3">
-        <f>C5*0.5</f>
-        <v>250</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="L3">
-        <f>K2</f>
-        <v>5000</v>
-      </c>
+        <f>G2</f>
+        <v>250</v>
+      </c>
+      <c r="J3" s="1"/>
     </row>
     <row r="5" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C5">
-        <f>D6</f>
         <v>500</v>
       </c>
       <c r="F5" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G5">
-        <f>H6</f>
-        <v>250</v>
-      </c>
-      <c r="J5" t="s">
-        <v>2</v>
-      </c>
-      <c r="K5">
-        <v>2000</v>
+        <v>250</v>
       </c>
     </row>
     <row r="6" spans="2:12" x14ac:dyDescent="0.25">
@@ -530,15 +594,10 @@
         <v>0</v>
       </c>
       <c r="H6">
-        <v>250</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L6">
-        <f>K5</f>
-        <v>2000</v>
-      </c>
+        <f>G5</f>
+        <v>250</v>
+      </c>
+      <c r="J6" s="1"/>
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
@@ -551,30 +610,28 @@
         <v>0</v>
       </c>
       <c r="G8">
-        <f>H9</f>
-        <v>500</v>
+        <v>250</v>
       </c>
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B9" s="1" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D9">
-        <f>G5/0.5</f>
+        <f>C5</f>
         <v>500</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H9">
-        <f>C13*0.5</f>
-        <v>500</v>
+        <v>250</v>
       </c>
       <c r="J9" s="1"/>
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B10" s="1" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D10">
         <f>C8-D9</f>
@@ -583,53 +640,54 @@
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.25">
       <c r="F11" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G11">
-        <v>200</v>
+        <v>250</v>
       </c>
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C12">
-        <v>50</v>
+        <v>500</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="H12">
-        <f>G11</f>
-        <v>200</v>
+        <v>250</v>
       </c>
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B13" t="s">
-        <v>2</v>
-      </c>
-      <c r="C13">
-        <v>1000</v>
+      <c r="B13" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D13">
+        <f>C12</f>
+        <v>500</v>
       </c>
     </row>
     <row r="14" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B14" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D14">
-        <f>SUM(C12:C13)</f>
-        <v>1050</v>
-      </c>
+      <c r="B14" s="1"/>
       <c r="F14" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G14">
-        <v>50</v>
+        <f>H9</f>
+        <v>250</v>
       </c>
     </row>
     <row r="15" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B15" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C15">
+        <v>900</v>
+      </c>
       <c r="F15" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G15">
         <v>250</v>
@@ -640,73 +698,45 @@
         <v>8</v>
       </c>
       <c r="C16">
-        <f>D17</f>
-        <v>400</v>
+        <f>SUM(D17:D18)-C15</f>
+        <v>50</v>
       </c>
       <c r="F16" s="1" t="s">
         <v>0</v>
       </c>
       <c r="H16">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="17" spans="2:8" x14ac:dyDescent="0.25">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="17" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B17" s="1" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D17">
-        <f>G11*2</f>
-        <v>400</v>
-      </c>
-    </row>
-    <row r="18" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="F18" t="s">
-        <v>0</v>
-      </c>
-      <c r="G18">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="19" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B19" t="s">
-        <v>9</v>
-      </c>
-      <c r="C19">
-        <f>D20</f>
-        <v>100</v>
-      </c>
-      <c r="F19" t="s">
-        <v>11</v>
-      </c>
-      <c r="H19">
-        <f>G18-H20</f>
-        <v>150</v>
-      </c>
-    </row>
-    <row r="20" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B20" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D20">
-        <f>G14*2</f>
-        <v>100</v>
-      </c>
-      <c r="F20" t="s">
-        <v>2</v>
-      </c>
-      <c r="H20">
-        <f>G15*(K5/L3)</f>
-        <v>100</v>
-      </c>
+        <f>C12</f>
+        <v>500</v>
+      </c>
+    </row>
+    <row r="18" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B18" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D18">
+        <f>C15*(G15/SUM(G14:G15))</f>
+        <v>450</v>
+      </c>
+    </row>
+    <row r="20" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B20" s="1"/>
     </row>
     <row r="34" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B34" t="str" cm="1">
-        <f t="array" ref="B34:B40">_xlfn.LET(_xlpm.x,_xlfn.UNIQUE(B$2:B$33),_xlfn._xlws.FILTER(_xlpm.x,_xlpm.x&lt;&gt;0))</f>
+        <f t="array" ref="B34:B38">_xlfn.LET(_xlpm.x,_xlfn.UNIQUE(B$2:B$33),_xlfn._xlws.FILTER(_xlpm.x,_xlpm.x&lt;&gt;0))</f>
         <v>Cash</v>
       </c>
       <c r="D34" cm="1">
         <f t="array" ref="D34">SUMPRODUCT(--(B34=B$2:B$33),C$2:C$33-D$2:D$33)</f>
-        <v>0</v>
+        <v>1450</v>
       </c>
       <c r="F34" t="str" cm="1">
         <f t="array" ref="F34:F36">_xlfn.LET(_xlpm.x,_xlfn.UNIQUE(F$2:F$33),_xlfn._xlws.FILTER(_xlpm.x,_xlpm.x&lt;&gt;0))</f>
@@ -714,15 +744,15 @@
       </c>
       <c r="H34" cm="1">
         <f t="array" ref="H34">SUMPRODUCT(--(F34=F$2:F$33),G$2:G$33-H$2:H$33)</f>
-        <v>250</v>
-      </c>
-      <c r="J34" t="str" cm="1">
-        <f t="array" ref="J34:J35">_xlfn.LET(_xlpm.x,_xlfn.UNIQUE(J$2:J$33),_xlfn._xlws.FILTER(_xlpm.x,_xlpm.x&lt;&gt;0))</f>
-        <v>Inventory</v>
-      </c>
-      <c r="L34" cm="1">
+        <v>0</v>
+      </c>
+      <c r="J34" t="e" cm="1" vm="1">
+        <f t="array" ref="J34">_xlfn.LET(_xlpm.x,_xlfn.UNIQUE(J$2:J$33),_xlfn._xlws.FILTER(_xlpm.x,_xlpm.x&lt;&gt;0))</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="L34" t="e" cm="1" vm="2">
         <f t="array" ref="L34">SUMPRODUCT(--(J34=J$2:J$33),K$2:K$33-L$2:L$33)</f>
-        <v>3000</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="35" spans="2:12" x14ac:dyDescent="0.25">
@@ -738,14 +768,11 @@
       </c>
       <c r="H35" cm="1">
         <f t="array" ref="H35">SUMPRODUCT(--(F35=F$2:F$33),G$2:G$33-H$2:H$33)</f>
-        <v>-100</v>
-      </c>
-      <c r="J35" t="str">
-        <v>Net Transfers</v>
+        <v>250</v>
       </c>
       <c r="L35" cm="1">
         <f t="array" ref="L35">SUMPRODUCT(--(J35=J$2:J$33),K$2:K$33-L$2:L$33)</f>
-        <v>-3000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36" spans="2:12" x14ac:dyDescent="0.25">
@@ -754,14 +781,14 @@
       </c>
       <c r="D36" cm="1">
         <f t="array" ref="D36">SUMPRODUCT(--(B36=B$2:B$33),C$2:C$33-D$2:D$33)</f>
-        <v>500</v>
+        <v>-450</v>
       </c>
       <c r="F36" t="str">
-        <v>Profit from Sale of Inventory</v>
+        <v>Accounts Payable</v>
       </c>
       <c r="H36" cm="1">
         <f t="array" ref="H36">SUMPRODUCT(--(F36=F$2:F$33),G$2:G$33-H$2:H$33)</f>
-        <v>-150</v>
+        <v>-250</v>
       </c>
       <c r="L36" cm="1">
         <f t="array" ref="L36">SUMPRODUCT(--(J36=J$2:J$33),K$2:K$33-L$2:L$33)</f>
@@ -770,7 +797,7 @@
     </row>
     <row r="37" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B37" t="str">
-        <v>Capital Gains or Losses</v>
+        <v>Capital Gains</v>
       </c>
       <c r="D37" cm="1">
         <f t="array" ref="D37">SUMPRODUCT(--(B37=B$2:B$33),C$2:C$33-D$2:D$33)</f>
@@ -787,7 +814,7 @@
     </row>
     <row r="38" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B38" t="str">
-        <v>Exchange Expense</v>
+        <v>Capital Loss</v>
       </c>
       <c r="D38" cm="1">
         <f t="array" ref="D38">SUMPRODUCT(--(B38=B$2:B$33),C$2:C$33-D$2:D$33)</f>
@@ -803,12 +830,9 @@
       </c>
     </row>
     <row r="39" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B39" t="str">
-        <v>Rent Expense</v>
-      </c>
       <c r="D39" cm="1">
         <f t="array" ref="D39">SUMPRODUCT(--(B39=B$2:B$33),C$2:C$33-D$2:D$33)</f>
-        <v>400</v>
+        <v>0</v>
       </c>
       <c r="H39" cm="1">
         <f t="array" ref="H39">SUMPRODUCT(--(F39=F$2:F$33),G$2:G$33-H$2:H$33)</f>
@@ -820,12 +844,9 @@
       </c>
     </row>
     <row r="40" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B40" t="str">
-        <v>Spoilage Expense</v>
-      </c>
       <c r="D40" cm="1">
         <f t="array" ref="D40">SUMPRODUCT(--(B40=B$2:B$33),C$2:C$33-D$2:D$33)</f>
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="H40" cm="1">
         <f t="array" ref="H40">SUMPRODUCT(--(F40=F$2:F$33),G$2:G$33-H$2:H$33)</f>

</xml_diff>

<commit_message>
refactor!: introduce TransactionMaterial and semantic transaction groups
- introduce TransactionMaterial and TransactionMaterialFactory abstractions
- make Transaction, ExchangeTransactions, and TerminalTransactions first-class transaction material
- replace anonymous wrapper groups with semantic transaction bundles
- simplify EventBuilder to record resolutions and transaction material directly
- distinguish ordered groups from semantic transaction groups
- eliminate .toGroup() conversions throughout the codebase
- preserve deterministic transaction ordering while retaining semantic structure
- expand tests for transaction material, semantic groups, and event construction
</commit_message>
<xml_diff>
--- a/example/account-ledger.xlsx
+++ b/example/account-ledger.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Local Storage\Repositories\Finance\Lattice\example\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73C0B67D-8071-4D6A-8DBE-5F5E29633735}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B1F8EDC-CA21-4E00-95C6-696770FF1623}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="52005" yWindow="4050" windowWidth="18285" windowHeight="14550" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9555" yWindow="3015" windowWidth="18285" windowHeight="10980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -83,7 +83,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="14">
   <si>
     <t>Cash</t>
   </si>
@@ -100,16 +100,31 @@
     <t>C (Inventory)</t>
   </si>
   <si>
-    <t>Net Transfers</t>
-  </si>
-  <si>
-    <t>Capital Gains</t>
-  </si>
-  <si>
     <t>Accounts Payable</t>
   </si>
   <si>
-    <t>Capital Loss</t>
+    <t>Transfers to USD</t>
+  </si>
+  <si>
+    <t>Capital Gains from Disposition of A</t>
+  </si>
+  <si>
+    <t>Transfers to B</t>
+  </si>
+  <si>
+    <t>Capital Gains from Disposition of B</t>
+  </si>
+  <si>
+    <t>Capital Loss from Disposition of B</t>
+  </si>
+  <si>
+    <t>Transfers from B</t>
+  </si>
+  <si>
+    <t>Transfers from A</t>
+  </si>
+  <si>
+    <t>Transfers to A</t>
   </si>
 </sst>
 </file>
@@ -561,7 +576,7 @@
         <v>1000</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="H3">
         <f>G2</f>
@@ -571,13 +586,13 @@
     </row>
     <row r="5" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C5">
         <v>500</v>
       </c>
       <c r="F5" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="G5">
         <v>250</v>
@@ -615,14 +630,14 @@
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B9" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D9">
         <f>C5</f>
         <v>500</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="H9">
         <v>250</v>
@@ -631,7 +646,7 @@
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B10" s="1" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D10">
         <f>C8-D9</f>
@@ -648,13 +663,13 @@
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C12">
         <v>500</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H12">
         <v>250</v>
@@ -672,7 +687,7 @@
     <row r="14" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B14" s="1"/>
       <c r="F14" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="G14">
         <f>H9</f>
@@ -687,7 +702,7 @@
         <v>900</v>
       </c>
       <c r="F15" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="G15">
         <v>250</v>
@@ -695,7 +710,7 @@
     </row>
     <row r="16" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C16">
         <f>SUM(D17:D18)-C15</f>
@@ -708,43 +723,96 @@
         <v>500</v>
       </c>
     </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B17" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D17">
         <f>C12</f>
         <v>500</v>
       </c>
     </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B18" s="1" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="D18">
         <f>C15*(G15/SUM(G14:G15))</f>
         <v>450</v>
       </c>
-    </row>
-    <row r="20" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B20" s="1"/>
+      <c r="F18" t="s">
+        <v>0</v>
+      </c>
+      <c r="G18">
+        <f>D22/2</f>
+        <v>725</v>
+      </c>
+    </row>
+    <row r="19" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="F19" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G19">
+        <f>SUM(H20:H21)-G18</f>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="20" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B20" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C20">
+        <f>D18</f>
+        <v>450</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H20">
+        <f>G15</f>
+        <v>250</v>
+      </c>
+    </row>
+    <row r="21" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B21" t="s">
+        <v>8</v>
+      </c>
+      <c r="C21">
+        <f>D22-C20</f>
+        <v>1000</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H21">
+        <f>G18*(C21/SUM(C20:C21))</f>
+        <v>500.00000000000006</v>
+      </c>
+    </row>
+    <row r="22" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B22" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D22">
+        <v>1450</v>
+      </c>
     </row>
     <row r="34" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B34" t="str" cm="1">
-        <f t="array" ref="B34:B38">_xlfn.LET(_xlpm.x,_xlfn.UNIQUE(B$2:B$33),_xlfn._xlws.FILTER(_xlpm.x,_xlpm.x&lt;&gt;0))</f>
+        <f t="array" ref="B34:B40">_xlfn.LET(_xlpm.x,_xlfn.UNIQUE(B$2:B$33),_xlfn._xlws.FILTER(_xlpm.x,_xlpm.x&lt;&gt;0))</f>
         <v>Cash</v>
       </c>
       <c r="D34" cm="1">
         <f t="array" ref="D34">SUMPRODUCT(--(B34=B$2:B$33),C$2:C$33-D$2:D$33)</f>
-        <v>1450</v>
+        <v>0</v>
       </c>
       <c r="F34" t="str" cm="1">
-        <f t="array" ref="F34:F36">_xlfn.LET(_xlpm.x,_xlfn.UNIQUE(F$2:F$33),_xlfn._xlws.FILTER(_xlpm.x,_xlpm.x&lt;&gt;0))</f>
+        <f t="array" ref="F34:F38">_xlfn.LET(_xlpm.x,_xlfn.UNIQUE(F$2:F$33),_xlfn._xlws.FILTER(_xlpm.x,_xlpm.x&lt;&gt;0))</f>
         <v>Cash</v>
       </c>
       <c r="H34" cm="1">
         <f t="array" ref="H34">SUMPRODUCT(--(F34=F$2:F$33),G$2:G$33-H$2:H$33)</f>
-        <v>0</v>
+        <v>725</v>
       </c>
       <c r="J34" t="e" cm="1" vm="1">
         <f t="array" ref="J34">_xlfn.LET(_xlpm.x,_xlfn.UNIQUE(J$2:J$33),_xlfn._xlws.FILTER(_xlpm.x,_xlpm.x&lt;&gt;0))</f>
@@ -764,11 +832,11 @@
         <v>-1000</v>
       </c>
       <c r="F35" t="str">
-        <v>Net Transfers</v>
+        <v>Transfers from A</v>
       </c>
       <c r="H35" cm="1">
         <f t="array" ref="H35">SUMPRODUCT(--(F35=F$2:F$33),G$2:G$33-H$2:H$33)</f>
-        <v>250</v>
+        <v>-500.00000000000006</v>
       </c>
       <c r="L35" cm="1">
         <f t="array" ref="L35">SUMPRODUCT(--(J35=J$2:J$33),K$2:K$33-L$2:L$33)</f>
@@ -777,11 +845,11 @@
     </row>
     <row r="36" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B36" t="str">
-        <v>Net Transfers</v>
+        <v>Transfers to B</v>
       </c>
       <c r="D36" cm="1">
         <f t="array" ref="D36">SUMPRODUCT(--(B36=B$2:B$33),C$2:C$33-D$2:D$33)</f>
-        <v>-450</v>
+        <v>500</v>
       </c>
       <c r="F36" t="str">
         <v>Accounts Payable</v>
@@ -797,12 +865,15 @@
     </row>
     <row r="37" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B37" t="str">
-        <v>Capital Gains</v>
+        <v>Capital Gains from Disposition of B</v>
       </c>
       <c r="D37" cm="1">
         <f t="array" ref="D37">SUMPRODUCT(--(B37=B$2:B$33),C$2:C$33-D$2:D$33)</f>
         <v>-50</v>
       </c>
+      <c r="F37" t="str">
+        <v>Transfers to A</v>
+      </c>
       <c r="H37" cm="1">
         <f t="array" ref="H37">SUMPRODUCT(--(F37=F$2:F$33),G$2:G$33-H$2:H$33)</f>
         <v>0</v>
@@ -814,15 +885,18 @@
     </row>
     <row r="38" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B38" t="str">
-        <v>Capital Loss</v>
+        <v>Transfers to USD</v>
       </c>
       <c r="D38" cm="1">
         <f t="array" ref="D38">SUMPRODUCT(--(B38=B$2:B$33),C$2:C$33-D$2:D$33)</f>
-        <v>50</v>
+        <v>500</v>
+      </c>
+      <c r="F38" t="str">
+        <v>Capital Gains from Disposition of A</v>
       </c>
       <c r="H38" cm="1">
         <f t="array" ref="H38">SUMPRODUCT(--(F38=F$2:F$33),G$2:G$33-H$2:H$33)</f>
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="L38" cm="1">
         <f t="array" ref="L38">SUMPRODUCT(--(J38=J$2:J$33),K$2:K$33-L$2:L$33)</f>
@@ -830,9 +904,12 @@
       </c>
     </row>
     <row r="39" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B39" t="str">
+        <v>Capital Loss from Disposition of B</v>
+      </c>
       <c r="D39" cm="1">
         <f t="array" ref="D39">SUMPRODUCT(--(B39=B$2:B$33),C$2:C$33-D$2:D$33)</f>
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="H39" cm="1">
         <f t="array" ref="H39">SUMPRODUCT(--(F39=F$2:F$33),G$2:G$33-H$2:H$33)</f>
@@ -844,6 +921,9 @@
       </c>
     </row>
     <row r="40" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B40" t="str">
+        <v>Transfers from B</v>
+      </c>
       <c r="D40" cm="1">
         <f t="array" ref="D40">SUMPRODUCT(--(B40=B$2:B$33),C$2:C$33-D$2:D$33)</f>
         <v>0</v>

</xml_diff>